<commit_message>
Add main.py and update project documents
Add new main.py and update binary project documents (Documentation.docx, LAM_Jimmy-planning-initial-TPI.xlsx). Two Office temporary files (~$cumentation.docx, ~WRL0789.tmp) were also added — likely editor temp files; consider removing them and adding appropriate patterns to .gitignore if they were committed unintentionally.
</commit_message>
<xml_diff>
--- a/Documents/LAM_Jimmy-planning-initial-TPI.xlsx
+++ b/Documents/LAM_Jimmy-planning-initial-TPI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk74hjc\Desktop\TPI\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BC653B-103B-40AD-918D-A2CC11AC8500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C86845-FD20-4D07-AA56-0D5F9BD38B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -808,6 +808,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="29" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -820,6 +847,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -833,36 +863,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="29" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -939,8 +939,8 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FF65D5CD"/>
       <color rgb="FF42ACD2"/>
-      <color rgb="FF65D5CD"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1144,62 +1144,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53"/>
+      <c r="T1" s="53"/>
+      <c r="U1" s="53"/>
+      <c r="V1" s="53"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="53"/>
     </row>
     <row r="2" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="U2" s="56"/>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="56"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="54"/>
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
+      <c r="V2" s="54"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="54"/>
+      <c r="Y2" s="54"/>
     </row>
     <row r="3" spans="1:25" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1207,37 +1207,37 @@
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="45" t="s">
+      <c r="E4" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="F4" s="45"/>
-      <c r="G4" s="46" t="s">
+      <c r="F4" s="55"/>
+      <c r="G4" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="47" t="s">
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="48" t="s">
+      <c r="M4" s="57"/>
+      <c r="N4" s="57"/>
+      <c r="O4" s="57"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="48"/>
-      <c r="S4" s="48"/>
-      <c r="T4" s="48"/>
-      <c r="U4" s="48"/>
-      <c r="V4" s="49" t="s">
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="W4" s="49"/>
-      <c r="X4" s="49"/>
-      <c r="Y4" s="49"/>
+      <c r="W4" s="59"/>
+      <c r="X4" s="59"/>
+      <c r="Y4" s="59"/>
     </row>
     <row r="5" spans="1:25" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -1317,12 +1317,12 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
+      <c r="B6" s="50"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
       <c r="E6" s="7" t="s">
         <v>31</v>
       </c>
@@ -1388,12 +1388,12 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="E7" s="11" t="s">
         <v>31</v>
       </c>
@@ -1447,33 +1447,33 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="42"/>
-      <c r="M8" s="42"/>
-      <c r="N8" s="42"/>
-      <c r="O8" s="42"/>
-      <c r="P8" s="42"/>
-      <c r="Q8" s="42"/>
-      <c r="R8" s="42"/>
-      <c r="S8" s="42"/>
-      <c r="T8" s="42"/>
-      <c r="U8" s="42"/>
-      <c r="V8" s="42"/>
-      <c r="W8" s="42"/>
-      <c r="X8" s="42"/>
-      <c r="Y8" s="42"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
+      <c r="J8" s="51"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="51"/>
+      <c r="O8" s="51"/>
+      <c r="P8" s="51"/>
+      <c r="Q8" s="51"/>
+      <c r="R8" s="51"/>
+      <c r="S8" s="51"/>
+      <c r="T8" s="51"/>
+      <c r="U8" s="51"/>
+      <c r="V8" s="51"/>
+      <c r="W8" s="51"/>
+      <c r="X8" s="51"/>
+      <c r="Y8" s="51"/>
     </row>
     <row r="9" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14">
@@ -1526,7 +1526,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="26"/>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="39" t="s">
         <v>54</v>
       </c>
       <c r="G10" s="19"/>
@@ -1587,33 +1587,33 @@
       <c r="Y11" s="20"/>
     </row>
     <row r="12" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="43"/>
-      <c r="R12" s="43"/>
-      <c r="S12" s="43"/>
-      <c r="T12" s="43"/>
-      <c r="U12" s="43"/>
-      <c r="V12" s="43"/>
-      <c r="W12" s="43"/>
-      <c r="X12" s="43"/>
-      <c r="Y12" s="43"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="52"/>
+      <c r="M12" s="52"/>
+      <c r="N12" s="52"/>
+      <c r="O12" s="52"/>
+      <c r="P12" s="52"/>
+      <c r="Q12" s="52"/>
+      <c r="R12" s="52"/>
+      <c r="S12" s="52"/>
+      <c r="T12" s="52"/>
+      <c r="U12" s="52"/>
+      <c r="V12" s="52"/>
+      <c r="W12" s="52"/>
+      <c r="X12" s="52"/>
+      <c r="Y12" s="52"/>
     </row>
     <row r="13" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14">
@@ -1629,7 +1629,7 @@
         <v>3.5</v>
       </c>
       <c r="E13" s="20"/>
-      <c r="F13" s="57" t="s">
+      <c r="F13" s="41" t="s">
         <v>54</v>
       </c>
       <c r="G13" s="29"/>
@@ -1838,33 +1838,33 @@
       <c r="Y18" s="20"/>
     </row>
     <row r="19" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="50"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="Q19" s="50"/>
-      <c r="R19" s="50"/>
-      <c r="S19" s="50"/>
-      <c r="T19" s="50"/>
-      <c r="U19" s="50"/>
-      <c r="V19" s="50"/>
-      <c r="W19" s="50"/>
-      <c r="X19" s="50"/>
-      <c r="Y19" s="50"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44"/>
+      <c r="K19" s="44"/>
+      <c r="L19" s="44"/>
+      <c r="M19" s="44"/>
+      <c r="N19" s="44"/>
+      <c r="O19" s="44"/>
+      <c r="P19" s="44"/>
+      <c r="Q19" s="44"/>
+      <c r="R19" s="44"/>
+      <c r="S19" s="44"/>
+      <c r="T19" s="44"/>
+      <c r="U19" s="44"/>
+      <c r="V19" s="44"/>
+      <c r="W19" s="44"/>
+      <c r="X19" s="44"/>
+      <c r="Y19" s="44"/>
     </row>
     <row r="20" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
@@ -1945,22 +1945,22 @@
         <v>12</v>
       </c>
       <c r="B22" s="32"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="58"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="58"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
       <c r="I22" s="21"/>
-      <c r="J22" s="58"/>
-      <c r="K22" s="58"/>
-      <c r="L22" s="58"/>
-      <c r="M22" s="58"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="42"/>
+      <c r="L22" s="42"/>
+      <c r="M22" s="42"/>
       <c r="N22" s="21"/>
-      <c r="O22" s="58"/>
-      <c r="P22" s="58"/>
-      <c r="Q22" s="58"/>
-      <c r="R22" s="58"/>
+      <c r="O22" s="42"/>
+      <c r="P22" s="42"/>
+      <c r="Q22" s="42"/>
+      <c r="R22" s="42"/>
       <c r="S22" s="21"/>
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
@@ -1970,33 +1970,33 @@
       <c r="Y22" s="34"/>
     </row>
     <row r="23" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="55" t="s">
+      <c r="A23" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="55"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55"/>
-      <c r="K23" s="55"/>
-      <c r="L23" s="55"/>
-      <c r="M23" s="55"/>
-      <c r="N23" s="55"/>
-      <c r="O23" s="55"/>
-      <c r="P23" s="55"/>
-      <c r="Q23" s="55"/>
-      <c r="R23" s="55"/>
-      <c r="S23" s="55"/>
-      <c r="T23" s="55"/>
-      <c r="U23" s="55"/>
-      <c r="V23" s="55"/>
-      <c r="W23" s="55"/>
-      <c r="X23" s="55"/>
-      <c r="Y23" s="55"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="49"/>
+      <c r="N23" s="49"/>
+      <c r="O23" s="49"/>
+      <c r="P23" s="49"/>
+      <c r="Q23" s="49"/>
+      <c r="R23" s="49"/>
+      <c r="S23" s="49"/>
+      <c r="T23" s="49"/>
+      <c r="U23" s="49"/>
+      <c r="V23" s="49"/>
+      <c r="W23" s="49"/>
+      <c r="X23" s="49"/>
+      <c r="Y23" s="49"/>
     </row>
     <row r="24" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14">
@@ -2043,59 +2043,59 @@
       <c r="C25" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="D25" s="59">
+      <c r="D25" s="43">
         <v>1</v>
       </c>
-      <c r="E25" s="58"/>
-      <c r="F25" s="58"/>
-      <c r="G25" s="58"/>
-      <c r="H25" s="58"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
       <c r="I25" s="21"/>
-      <c r="J25" s="58"/>
-      <c r="K25" s="58"/>
-      <c r="L25" s="58"/>
-      <c r="M25" s="58"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="42"/>
       <c r="N25" s="21"/>
-      <c r="O25" s="58"/>
-      <c r="P25" s="58"/>
-      <c r="Q25" s="58"/>
-      <c r="R25" s="58"/>
+      <c r="O25" s="42"/>
+      <c r="P25" s="42"/>
+      <c r="Q25" s="42"/>
+      <c r="R25" s="42"/>
       <c r="S25" s="21"/>
       <c r="T25" s="22"/>
       <c r="U25" s="22"/>
-      <c r="V25" s="58"/>
-      <c r="W25" s="58"/>
+      <c r="V25" s="42"/>
+      <c r="W25" s="42"/>
       <c r="X25" s="21"/>
-      <c r="Y25" s="58"/>
+      <c r="Y25" s="42"/>
     </row>
     <row r="26" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="51" t="s">
+      <c r="A26" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="52"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="52"/>
-      <c r="P26" s="52"/>
-      <c r="Q26" s="52"/>
-      <c r="R26" s="52"/>
-      <c r="S26" s="52"/>
-      <c r="T26" s="52"/>
-      <c r="U26" s="52"/>
-      <c r="V26" s="52"/>
-      <c r="W26" s="52"/>
-      <c r="X26" s="52"/>
-      <c r="Y26" s="52"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="46"/>
+      <c r="K26" s="46"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="46"/>
+      <c r="Q26" s="46"/>
+      <c r="R26" s="46"/>
+      <c r="S26" s="46"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+      <c r="V26" s="46"/>
+      <c r="W26" s="46"/>
+      <c r="X26" s="46"/>
+      <c r="Y26" s="46"/>
     </row>
     <row r="27" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14">
@@ -2167,66 +2167,61 @@
       <c r="Y28" s="1"/>
     </row>
     <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="53"/>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="53"/>
-      <c r="J30" s="53"/>
-      <c r="K30" s="53"/>
-      <c r="L30" s="53"/>
-      <c r="M30" s="53"/>
-      <c r="N30" s="53"/>
-      <c r="O30" s="53"/>
-      <c r="P30" s="53"/>
-      <c r="Q30" s="53"/>
-      <c r="R30" s="53"/>
-      <c r="S30" s="53"/>
-      <c r="T30" s="53"/>
-      <c r="U30" s="53"/>
-      <c r="V30" s="53"/>
-      <c r="W30" s="53"/>
-      <c r="X30" s="53"/>
-      <c r="Y30" s="53"/>
+      <c r="A30" s="47"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="47"/>
+      <c r="D30" s="47"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="47"/>
+      <c r="L30" s="47"/>
+      <c r="M30" s="47"/>
+      <c r="N30" s="47"/>
+      <c r="O30" s="47"/>
+      <c r="P30" s="47"/>
+      <c r="Q30" s="47"/>
+      <c r="R30" s="47"/>
+      <c r="S30" s="47"/>
+      <c r="T30" s="47"/>
+      <c r="U30" s="47"/>
+      <c r="V30" s="47"/>
+      <c r="W30" s="47"/>
+      <c r="X30" s="47"/>
+      <c r="Y30" s="47"/>
     </row>
     <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="54"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="54"/>
-      <c r="H31" s="54"/>
-      <c r="I31" s="54"/>
-      <c r="J31" s="54"/>
-      <c r="K31" s="54"/>
-      <c r="L31" s="54"/>
-      <c r="M31" s="54"/>
-      <c r="N31" s="54"/>
-      <c r="O31" s="54"/>
-      <c r="P31" s="54"/>
-      <c r="Q31" s="54"/>
-      <c r="R31" s="54"/>
-      <c r="S31" s="54"/>
-      <c r="T31" s="54"/>
-      <c r="U31" s="54"/>
-      <c r="V31" s="54"/>
-      <c r="W31" s="54"/>
-      <c r="X31" s="54"/>
-      <c r="Y31" s="54"/>
+      <c r="A31" s="48"/>
+      <c r="B31" s="48"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="48"/>
+      <c r="H31" s="48"/>
+      <c r="I31" s="48"/>
+      <c r="J31" s="48"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="48"/>
+      <c r="M31" s="48"/>
+      <c r="N31" s="48"/>
+      <c r="O31" s="48"/>
+      <c r="P31" s="48"/>
+      <c r="Q31" s="48"/>
+      <c r="R31" s="48"/>
+      <c r="S31" s="48"/>
+      <c r="T31" s="48"/>
+      <c r="U31" s="48"/>
+      <c r="V31" s="48"/>
+      <c r="W31" s="48"/>
+      <c r="X31" s="48"/>
+      <c r="Y31" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A19:Y19"/>
-    <mergeCell ref="A26:Y26"/>
-    <mergeCell ref="A30:Y30"/>
-    <mergeCell ref="A31:Y31"/>
-    <mergeCell ref="A23:Y23"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A8:Y8"/>
@@ -2238,6 +2233,11 @@
     <mergeCell ref="L4:P4"/>
     <mergeCell ref="Q4:U4"/>
     <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="A19:Y19"/>
+    <mergeCell ref="A26:Y26"/>
+    <mergeCell ref="A30:Y30"/>
+    <mergeCell ref="A31:Y31"/>
+    <mergeCell ref="A23:Y23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>